<commit_message>
Auto sync Onetech 28/10/2026 13:30
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19848" uniqueCount="1349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19845" uniqueCount="1349">
   <si>
     <t>DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH</t>
   </si>
@@ -28783,14 +28783,14 @@
       <c r="P197" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="Q197" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="R197" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S197" s="3" t="s">
-        <v>46</v>
+      <c r="Q197" s="5">
+        <v>1</v>
+      </c>
+      <c r="R197" s="5">
+        <v>1</v>
+      </c>
+      <c r="S197" s="5">
+        <v>1</v>
       </c>
       <c r="T197" s="3" t="s">
         <v>46</v>

</xml_diff>

<commit_message>
Auto sync Onetech 28/10/2026 14:05
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -80909,13 +80909,13 @@
         <v>79</v>
       </c>
       <c r="Q614" s="5">
+        <v>27</v>
+      </c>
+      <c r="R614" s="5">
         <v>26</v>
       </c>
-      <c r="R614" s="5">
-        <v>25</v>
-      </c>
       <c r="S614" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="T614" s="3" t="s">
         <v>1172</v>

</xml_diff>

<commit_message>
Auto sync Onetech 30/10/2026 10:00
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -65139,13 +65139,13 @@
         <v>196</v>
       </c>
       <c r="Q487" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R487" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S487" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T487" s="3" t="s">
         <v>1207</v>
@@ -66889,13 +66889,13 @@
         <v>196</v>
       </c>
       <c r="Q501" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R501" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S501" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T501" s="3" t="s">
         <v>1207</v>
@@ -68514,13 +68514,13 @@
         <v>196</v>
       </c>
       <c r="Q514" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R514" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S514" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T514" s="3" t="s">
         <v>1207</v>
@@ -72264,13 +72264,13 @@
         <v>210</v>
       </c>
       <c r="Q544" s="5">
+        <v>4</v>
+      </c>
+      <c r="R544" s="5">
         <v>3</v>
       </c>
-      <c r="R544" s="5">
-        <v>2</v>
-      </c>
       <c r="S544" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T544" s="3" t="s">
         <v>1207</v>
@@ -74139,13 +74139,13 @@
         <v>196</v>
       </c>
       <c r="Q559" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R559" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S559" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T559" s="3" t="s">
         <v>1207</v>
@@ -76389,13 +76389,13 @@
         <v>196</v>
       </c>
       <c r="Q577" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R577" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="S577" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="T577" s="3" t="s">
         <v>1207</v>
@@ -80139,13 +80139,13 @@
         <v>196</v>
       </c>
       <c r="Q607" s="5">
+        <v>30</v>
+      </c>
+      <c r="R607" s="5">
         <v>29</v>
       </c>
-      <c r="R607" s="5">
-        <v>28</v>
-      </c>
       <c r="S607" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="T607" s="3" t="s">
         <v>1207</v>

</xml_diff>

<commit_message>
Auto sync Onetech 31/10/2026 21:45
</commit_message>
<xml_diff>
--- a/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
+++ b/data/Thang10/DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18937" uniqueCount="1341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18931" uniqueCount="1341">
   <si>
     <t>DANH_SACH_KET_QUA_CUA_HANG_THAM_GIA_CHUONG_TRINH</t>
   </si>
@@ -3388,6 +3388,21 @@
     <t>1039, Phạm Văn Đồng</t>
   </si>
   <si>
+    <t>3057973</t>
+  </si>
+  <si>
+    <t>Hùng Anh</t>
+  </si>
+  <si>
+    <t>23, Đường 100</t>
+  </si>
+  <si>
+    <t>3142121</t>
+  </si>
+  <si>
+    <t>Anh Đại</t>
+  </si>
+  <si>
     <t>2800</t>
   </si>
   <si>
@@ -3397,21 +3412,6 @@
     <t>18/27, Đại Học</t>
   </si>
   <si>
-    <t>3057973</t>
-  </si>
-  <si>
-    <t>Hùng Anh</t>
-  </si>
-  <si>
-    <t>23, Đường 100</t>
-  </si>
-  <si>
-    <t>3142121</t>
-  </si>
-  <si>
-    <t>Anh Đại</t>
-  </si>
-  <si>
     <t>5355</t>
   </si>
   <si>
@@ -3457,6 +3457,15 @@
     <t>Lầu 2 toà A1, Đại Học Quốc Tế</t>
   </si>
   <si>
+    <t>3057968</t>
+  </si>
+  <si>
+    <t>Anh Hùng ( Trái Cây )</t>
+  </si>
+  <si>
+    <t>71, Đình Phong Phú</t>
+  </si>
+  <si>
     <t>5028</t>
   </si>
   <si>
@@ -3466,15 +3475,6 @@
     <t xml:space="preserve">108, Đường 4 Đại Học Nông Lâm </t>
   </si>
   <si>
-    <t>3057968</t>
-  </si>
-  <si>
-    <t>Anh Hùng ( Trái Cây )</t>
-  </si>
-  <si>
-    <t>71, Đình Phong Phú</t>
-  </si>
-  <si>
     <t>2340641</t>
   </si>
   <si>
@@ -3514,6 +3514,15 @@
     <t>203, Man Thiện</t>
   </si>
   <si>
+    <t>3265</t>
+  </si>
+  <si>
+    <t>Thu Hiền</t>
+  </si>
+  <si>
+    <t>235, Tăng Nhơn Phú</t>
+  </si>
+  <si>
     <t>3638</t>
   </si>
   <si>
@@ -3529,15 +3538,6 @@
     <t>5, Ngô Quyền</t>
   </si>
   <si>
-    <t>3265</t>
-  </si>
-  <si>
-    <t>Thu Hiền</t>
-  </si>
-  <si>
-    <t>235, Tăng Nhơn Phú</t>
-  </si>
-  <si>
     <t>Mức 2 - Kệ Mô Hình</t>
   </si>
   <si>
@@ -3568,19 +3568,19 @@
     <t>MSC_Cuộc thi ảnh Đại sứ Ngành hàng Gia Vị_HCM_All2026_T10</t>
   </si>
   <si>
+    <t>2430771</t>
+  </si>
+  <si>
+    <t>Tạp Hóa Vinh Phát</t>
+  </si>
+  <si>
+    <t>208/6B, Đường 138</t>
+  </si>
+  <si>
     <t>2790031</t>
   </si>
   <si>
     <t>Cao Ốc Xanh</t>
-  </si>
-  <si>
-    <t>2430771</t>
-  </si>
-  <si>
-    <t>Tạp Hóa Vinh Phát</t>
-  </si>
-  <si>
-    <t>208/6B, Đường 138</t>
   </si>
   <si>
     <t>4107</t>
@@ -57861,28 +57861,28 @@
         <v>46</v>
       </c>
       <c r="I430" s="3" t="s">
-        <v>269</v>
+        <v>1125</v>
       </c>
       <c r="J430" s="3" t="s">
-        <v>270</v>
+        <v>1126</v>
       </c>
       <c r="K430" s="3" t="s">
-        <v>271</v>
+        <v>1127</v>
       </c>
       <c r="L430" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M430" s="3" t="s">
-        <v>137</v>
+        <v>51</v>
       </c>
       <c r="N430" s="3" t="s">
-        <v>138</v>
+        <v>52</v>
       </c>
       <c r="O430" s="3" t="s">
-        <v>139</v>
+        <v>53</v>
       </c>
       <c r="P430" s="3" t="s">
-        <v>140</v>
+        <v>54</v>
       </c>
       <c r="Q430" s="3" t="s">
         <v>46</v>
@@ -57945,7 +57945,7 @@
         <v>58</v>
       </c>
       <c r="AK430" s="6">
-        <v>46301.91933796296</v>
+        <v>46324.30341940973</v>
       </c>
       <c r="AL430" s="3" t="s">
         <v>46</v>
@@ -57957,7 +57957,7 @@
         <v>58</v>
       </c>
       <c r="AO430" s="6">
-        <v>46301.91933796296</v>
+        <v>46324.30341940973</v>
       </c>
     </row>
     <row r="431" spans="1:41" x14ac:dyDescent="0.25">
@@ -57986,28 +57986,28 @@
         <v>46</v>
       </c>
       <c r="I431" s="3" t="s">
-        <v>340</v>
+        <v>1128</v>
       </c>
       <c r="J431" s="3" t="s">
-        <v>341</v>
+        <v>1129</v>
       </c>
       <c r="K431" s="3" t="s">
-        <v>342</v>
+        <v>104</v>
       </c>
       <c r="L431" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M431" s="3" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="N431" s="3" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="O431" s="3" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="P431" s="3" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="Q431" s="3" t="s">
         <v>46</v>
@@ -58070,7 +58070,7 @@
         <v>58</v>
       </c>
       <c r="AK431" s="6">
-        <v>46307.90555991898</v>
+        <v>46301.91933796296</v>
       </c>
       <c r="AL431" s="3" t="s">
         <v>46</v>
@@ -58082,7 +58082,7 @@
         <v>58</v>
       </c>
       <c r="AO431" s="6">
-        <v>46307.90555991898</v>
+        <v>46301.91933796296</v>
       </c>
     </row>
     <row r="432" spans="1:41" x14ac:dyDescent="0.25">
@@ -58111,28 +58111,28 @@
         <v>46</v>
       </c>
       <c r="I432" s="3" t="s">
-        <v>1125</v>
+        <v>579</v>
       </c>
       <c r="J432" s="3" t="s">
-        <v>1126</v>
+        <v>580</v>
       </c>
       <c r="K432" s="3" t="s">
-        <v>1127</v>
+        <v>581</v>
       </c>
       <c r="L432" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M432" s="3" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="N432" s="3" t="s">
-        <v>115</v>
+        <v>162</v>
       </c>
       <c r="O432" s="3" t="s">
-        <v>116</v>
+        <v>163</v>
       </c>
       <c r="P432" s="3" t="s">
-        <v>117</v>
+        <v>164</v>
       </c>
       <c r="Q432" s="3" t="s">
         <v>46</v>
@@ -58236,28 +58236,28 @@
         <v>46</v>
       </c>
       <c r="I433" s="3" t="s">
-        <v>1128</v>
+        <v>340</v>
       </c>
       <c r="J433" s="3" t="s">
-        <v>1129</v>
+        <v>341</v>
       </c>
       <c r="K433" s="3" t="s">
-        <v>1130</v>
+        <v>342</v>
       </c>
       <c r="L433" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M433" s="3" t="s">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="N433" s="3" t="s">
-        <v>52</v>
+        <v>77</v>
       </c>
       <c r="O433" s="3" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="P433" s="3" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="Q433" s="3" t="s">
         <v>46</v>
@@ -58320,7 +58320,7 @@
         <v>58</v>
       </c>
       <c r="AK433" s="6">
-        <v>46324.30341940973</v>
+        <v>46307.90555991898</v>
       </c>
       <c r="AL433" s="3" t="s">
         <v>46</v>
@@ -58332,7 +58332,7 @@
         <v>58</v>
       </c>
       <c r="AO433" s="6">
-        <v>46324.30341940973</v>
+        <v>46307.90555991898</v>
       </c>
     </row>
     <row r="434" spans="1:41" x14ac:dyDescent="0.25">
@@ -58361,28 +58361,28 @@
         <v>46</v>
       </c>
       <c r="I434" s="3" t="s">
+        <v>1130</v>
+      </c>
+      <c r="J434" s="3" t="s">
         <v>1131</v>
       </c>
-      <c r="J434" s="3" t="s">
+      <c r="K434" s="3" t="s">
         <v>1132</v>
-      </c>
-      <c r="K434" s="3" t="s">
-        <v>104</v>
       </c>
       <c r="L434" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M434" s="3" t="s">
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="N434" s="3" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="O434" s="3" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="P434" s="3" t="s">
-        <v>92</v>
+        <v>117</v>
       </c>
       <c r="Q434" s="3" t="s">
         <v>46</v>
@@ -58486,28 +58486,28 @@
         <v>46</v>
       </c>
       <c r="I435" s="3" t="s">
-        <v>579</v>
+        <v>1133</v>
       </c>
       <c r="J435" s="3" t="s">
-        <v>580</v>
+        <v>1134</v>
       </c>
       <c r="K435" s="3" t="s">
-        <v>581</v>
+        <v>1135</v>
       </c>
       <c r="L435" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M435" s="3" t="s">
-        <v>161</v>
+        <v>200</v>
       </c>
       <c r="N435" s="3" t="s">
-        <v>162</v>
+        <v>201</v>
       </c>
       <c r="O435" s="3" t="s">
-        <v>163</v>
+        <v>202</v>
       </c>
       <c r="P435" s="3" t="s">
-        <v>164</v>
+        <v>203</v>
       </c>
       <c r="Q435" s="3" t="s">
         <v>46</v>
@@ -58570,7 +58570,7 @@
         <v>58</v>
       </c>
       <c r="AK435" s="6">
-        <v>46301.91933796296</v>
+        <v>46324.30341940973</v>
       </c>
       <c r="AL435" s="3" t="s">
         <v>46</v>
@@ -58582,7 +58582,7 @@
         <v>58</v>
       </c>
       <c r="AO435" s="6">
-        <v>46301.91933796296</v>
+        <v>46324.30341940973</v>
       </c>
     </row>
     <row r="436" spans="1:41" x14ac:dyDescent="0.25">
@@ -58608,31 +58608,31 @@
         <v>45</v>
       </c>
       <c r="H436" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I436" s="3" t="s">
-        <v>1133</v>
+        <v>1136</v>
       </c>
       <c r="J436" s="3" t="s">
-        <v>1134</v>
+        <v>1137</v>
       </c>
       <c r="K436" s="3" t="s">
-        <v>1135</v>
+        <v>1138</v>
       </c>
       <c r="L436" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M436" s="3" t="s">
-        <v>200</v>
+        <v>114</v>
       </c>
       <c r="N436" s="3" t="s">
-        <v>201</v>
+        <v>115</v>
       </c>
       <c r="O436" s="3" t="s">
-        <v>202</v>
+        <v>116</v>
       </c>
       <c r="P436" s="3" t="s">
-        <v>203</v>
+        <v>117</v>
       </c>
       <c r="Q436" s="3" t="s">
         <v>46</v>
@@ -58644,7 +58644,7 @@
         <v>46</v>
       </c>
       <c r="T436" s="3" t="s">
-        <v>46</v>
+        <v>1139</v>
       </c>
       <c r="U436" s="3" t="s">
         <v>46</v>
@@ -58661,41 +58661,41 @@
       <c r="Y436" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="Z436" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="AA436" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="AB436" s="3" t="s">
-        <v>46</v>
+      <c r="Z436" s="7">
+        <v>10</v>
+      </c>
+      <c r="AA436" s="7">
+        <v>11</v>
+      </c>
+      <c r="AB436" s="7">
+        <v>1</v>
       </c>
       <c r="AC436" s="3" t="s">
-        <v>46</v>
+        <v>1140</v>
       </c>
       <c r="AD436" s="3" t="s">
-        <v>46</v>
+        <v>1141</v>
       </c>
       <c r="AE436" s="3" t="s">
-        <v>46</v>
+        <v>1142</v>
       </c>
       <c r="AF436" s="3" t="s">
-        <v>46</v>
+        <v>1143</v>
       </c>
       <c r="AG436" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="AH436" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="AI436" s="3" t="s">
-        <v>46</v>
+        <v>1144</v>
+      </c>
+      <c r="AH436" s="7">
+        <v>1</v>
+      </c>
+      <c r="AI436" s="3">
+        <v>0</v>
       </c>
       <c r="AJ436" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AK436" s="6">
-        <v>46324.30341940973</v>
+        <v>46316.57381339121</v>
       </c>
       <c r="AL436" s="3" t="s">
         <v>46</v>
@@ -58707,7 +58707,7 @@
         <v>58</v>
       </c>
       <c r="AO436" s="6">
-        <v>46324.30341940973</v>
+        <v>46316.57381339121</v>
       </c>
     </row>
     <row r="437" spans="1:41" x14ac:dyDescent="0.25">
@@ -58736,13 +58736,13 @@
         <v>45</v>
       </c>
       <c r="I437" s="3" t="s">
-        <v>1136</v>
+        <v>1145</v>
       </c>
       <c r="J437" s="3" t="s">
-        <v>1137</v>
+        <v>1146</v>
       </c>
       <c r="K437" s="3" t="s">
-        <v>1138</v>
+        <v>1147</v>
       </c>
       <c r="L437" s="3" t="s">
         <v>50</v>
@@ -58790,7 +58790,7 @@
         <v>10</v>
       </c>
       <c r="AA437" s="7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AB437" s="7">
         <v>1</v>
@@ -58820,7 +58820,7 @@
         <v>58</v>
       </c>
       <c r="AK437" s="6">
-        <v>46316.57381339121</v>
+        <v>46303.59298695602</v>
       </c>
       <c r="AL437" s="3" t="s">
         <v>46</v>
@@ -58832,7 +58832,7 @@
         <v>58</v>
       </c>
       <c r="AO437" s="6">
-        <v>46316.57381339121</v>
+        <v>46303.59298695602</v>
       </c>
     </row>
     <row r="438" spans="1:41" x14ac:dyDescent="0.25">
@@ -58861,28 +58861,28 @@
         <v>45</v>
       </c>
       <c r="I438" s="3" t="s">
-        <v>1145</v>
+        <v>1148</v>
       </c>
       <c r="J438" s="3" t="s">
-        <v>1146</v>
+        <v>1149</v>
       </c>
       <c r="K438" s="3" t="s">
-        <v>1147</v>
+        <v>1150</v>
       </c>
       <c r="L438" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M438" s="3" t="s">
-        <v>114</v>
+        <v>193</v>
       </c>
       <c r="N438" s="3" t="s">
-        <v>115</v>
+        <v>194</v>
       </c>
       <c r="O438" s="3" t="s">
-        <v>116</v>
+        <v>195</v>
       </c>
       <c r="P438" s="3" t="s">
-        <v>117</v>
+        <v>196</v>
       </c>
       <c r="Q438" s="3" t="s">
         <v>46</v>
@@ -58915,7 +58915,7 @@
         <v>10</v>
       </c>
       <c r="AA438" s="7">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AB438" s="7">
         <v>1</v>
@@ -58945,7 +58945,7 @@
         <v>58</v>
       </c>
       <c r="AK438" s="6">
-        <v>46303.59298695602</v>
+        <v>46307.90555991898</v>
       </c>
       <c r="AL438" s="3" t="s">
         <v>46</v>
@@ -58957,7 +58957,7 @@
         <v>58</v>
       </c>
       <c r="AO438" s="6">
-        <v>46303.59298695602</v>
+        <v>46307.90555991898</v>
       </c>
     </row>
     <row r="439" spans="1:41" x14ac:dyDescent="0.25">
@@ -58986,13 +58986,13 @@
         <v>45</v>
       </c>
       <c r="I439" s="3" t="s">
-        <v>1148</v>
+        <v>1151</v>
       </c>
       <c r="J439" s="3" t="s">
-        <v>1149</v>
+        <v>1152</v>
       </c>
       <c r="K439" s="3" t="s">
-        <v>1150</v>
+        <v>1153</v>
       </c>
       <c r="L439" s="3" t="s">
         <v>50</v>
@@ -59111,13 +59111,13 @@
         <v>45</v>
       </c>
       <c r="I440" s="3" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
       <c r="J440" s="3" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="K440" s="3" t="s">
-        <v>1153</v>
+        <v>1156</v>
       </c>
       <c r="L440" s="3" t="s">
         <v>50</v>
@@ -59165,10 +59165,10 @@
         <v>10</v>
       </c>
       <c r="AA440" s="7">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="AB440" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC440" s="3" t="s">
         <v>1140</v>
@@ -59186,7 +59186,7 @@
         <v>1144</v>
       </c>
       <c r="AH440" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI440" s="3">
         <v>0</v>
@@ -59195,7 +59195,7 @@
         <v>58</v>
       </c>
       <c r="AK440" s="6">
-        <v>46307.90555991898</v>
+        <v>46301.91933796296</v>
       </c>
       <c r="AL440" s="3" t="s">
         <v>46</v>
@@ -59207,7 +59207,7 @@
         <v>58</v>
       </c>
       <c r="AO440" s="6">
-        <v>46307.90555991898</v>
+        <v>46301.91933796296</v>
       </c>
     </row>
     <row r="441" spans="1:41" x14ac:dyDescent="0.25">
@@ -59236,28 +59236,28 @@
         <v>45</v>
       </c>
       <c r="I441" s="3" t="s">
-        <v>1154</v>
+        <v>233</v>
       </c>
       <c r="J441" s="3" t="s">
-        <v>1155</v>
+        <v>234</v>
       </c>
       <c r="K441" s="3" t="s">
-        <v>1156</v>
+        <v>235</v>
       </c>
       <c r="L441" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M441" s="3" t="s">
-        <v>193</v>
+        <v>154</v>
       </c>
       <c r="N441" s="3" t="s">
-        <v>194</v>
+        <v>155</v>
       </c>
       <c r="O441" s="3" t="s">
-        <v>195</v>
+        <v>156</v>
       </c>
       <c r="P441" s="3" t="s">
-        <v>196</v>
+        <v>157</v>
       </c>
       <c r="Q441" s="3" t="s">
         <v>46</v>
@@ -59290,10 +59290,10 @@
         <v>10</v>
       </c>
       <c r="AA441" s="7">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="AB441" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC441" s="3" t="s">
         <v>1140</v>
@@ -59311,7 +59311,7 @@
         <v>1144</v>
       </c>
       <c r="AH441" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI441" s="3">
         <v>0</v>
@@ -59361,28 +59361,28 @@
         <v>45</v>
       </c>
       <c r="I442" s="3" t="s">
-        <v>233</v>
+        <v>269</v>
       </c>
       <c r="J442" s="3" t="s">
-        <v>234</v>
+        <v>270</v>
       </c>
       <c r="K442" s="3" t="s">
-        <v>235</v>
+        <v>271</v>
       </c>
       <c r="L442" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M442" s="3" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="N442" s="3" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="O442" s="3" t="s">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="P442" s="3" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="Q442" s="3" t="s">
         <v>46</v>
@@ -59415,7 +59415,7 @@
         <v>10</v>
       </c>
       <c r="AA442" s="7">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AB442" s="7">
         <v>1</v>
@@ -59748,25 +59748,25 @@
         <v>50</v>
       </c>
       <c r="M445" s="3" t="s">
-        <v>62</v>
+        <v>193</v>
       </c>
       <c r="N445" s="3" t="s">
-        <v>63</v>
+        <v>194</v>
       </c>
       <c r="O445" s="3" t="s">
-        <v>64</v>
+        <v>195</v>
       </c>
       <c r="P445" s="3" t="s">
-        <v>65</v>
+        <v>196</v>
       </c>
       <c r="Q445" s="5">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="R445" s="5">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="S445" s="5">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="T445" s="3" t="s">
         <v>1139</v>
@@ -59790,7 +59790,7 @@
         <v>46</v>
       </c>
       <c r="AA445" s="7">
-        <v>1147670</v>
+        <v>199584</v>
       </c>
       <c r="AB445" s="7">
         <v>31</v>
@@ -59864,34 +59864,34 @@
         <v>1170</v>
       </c>
       <c r="J446" s="3" t="s">
-        <v>627</v>
+        <v>1171</v>
       </c>
       <c r="K446" s="3" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="L446" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M446" s="3" t="s">
-        <v>207</v>
+        <v>62</v>
       </c>
       <c r="N446" s="3" t="s">
-        <v>208</v>
+        <v>63</v>
       </c>
       <c r="O446" s="3" t="s">
-        <v>209</v>
+        <v>64</v>
       </c>
       <c r="P446" s="3" t="s">
-        <v>210</v>
+        <v>65</v>
       </c>
       <c r="Q446" s="5">
-        <v>4</v>
-      </c>
-      <c r="R446" s="3">
-        <v>0</v>
+        <v>25</v>
+      </c>
+      <c r="R446" s="5">
+        <v>25</v>
       </c>
       <c r="S446" s="5">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="T446" s="3" t="s">
         <v>1139</v>
@@ -59915,7 +59915,7 @@
         <v>46</v>
       </c>
       <c r="AA446" s="7">
-        <v>399168</v>
+        <v>1147670</v>
       </c>
       <c r="AB446" s="7">
         <v>31</v>
@@ -59986,37 +59986,37 @@
         <v>1160</v>
       </c>
       <c r="I447" s="3" t="s">
-        <v>1075</v>
+        <v>1173</v>
       </c>
       <c r="J447" s="3" t="s">
-        <v>1076</v>
+        <v>627</v>
       </c>
       <c r="K447" s="3" t="s">
-        <v>1077</v>
+        <v>1174</v>
       </c>
       <c r="L447" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M447" s="3" t="s">
-        <v>137</v>
+        <v>207</v>
       </c>
       <c r="N447" s="3" t="s">
-        <v>138</v>
+        <v>208</v>
       </c>
       <c r="O447" s="3" t="s">
-        <v>139</v>
+        <v>209</v>
       </c>
       <c r="P447" s="3" t="s">
-        <v>140</v>
+        <v>210</v>
       </c>
       <c r="Q447" s="5">
-        <v>12</v>
-      </c>
-      <c r="R447" s="5">
-        <v>10</v>
+        <v>4</v>
+      </c>
+      <c r="R447" s="3">
+        <v>0</v>
       </c>
       <c r="S447" s="5">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="T447" s="3" t="s">
         <v>1139</v>
@@ -60040,7 +60040,7 @@
         <v>46</v>
       </c>
       <c r="AA447" s="7">
-        <v>1133317</v>
+        <v>399168</v>
       </c>
       <c r="AB447" s="7">
         <v>31</v>
@@ -60111,37 +60111,37 @@
         <v>1160</v>
       </c>
       <c r="I448" s="3" t="s">
-        <v>1172</v>
+        <v>1075</v>
       </c>
       <c r="J448" s="3" t="s">
-        <v>1173</v>
+        <v>1076</v>
       </c>
       <c r="K448" s="3" t="s">
-        <v>1174</v>
+        <v>1077</v>
       </c>
       <c r="L448" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M448" s="3" t="s">
-        <v>193</v>
+        <v>137</v>
       </c>
       <c r="N448" s="3" t="s">
-        <v>194</v>
+        <v>138</v>
       </c>
       <c r="O448" s="3" t="s">
-        <v>195</v>
+        <v>139</v>
       </c>
       <c r="P448" s="3" t="s">
-        <v>196</v>
+        <v>140</v>
       </c>
       <c r="Q448" s="5">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="R448" s="5">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="S448" s="5">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="T448" s="3" t="s">
         <v>1139</v>
@@ -60165,7 +60165,7 @@
         <v>46</v>
       </c>
       <c r="AA448" s="7">
-        <v>199584</v>
+        <v>1133317</v>
       </c>
       <c r="AB448" s="7">
         <v>31</v>
@@ -60986,37 +60986,37 @@
         <v>1160</v>
       </c>
       <c r="I455" s="3" t="s">
-        <v>305</v>
+        <v>141</v>
       </c>
       <c r="J455" s="3" t="s">
-        <v>306</v>
+        <v>142</v>
       </c>
       <c r="K455" s="3" t="s">
-        <v>307</v>
+        <v>143</v>
       </c>
       <c r="L455" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M455" s="3" t="s">
-        <v>161</v>
+        <v>62</v>
       </c>
       <c r="N455" s="3" t="s">
-        <v>162</v>
+        <v>63</v>
       </c>
       <c r="O455" s="3" t="s">
-        <v>163</v>
+        <v>64</v>
       </c>
       <c r="P455" s="3" t="s">
-        <v>164</v>
+        <v>65</v>
       </c>
       <c r="Q455" s="5">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="R455" s="5">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="S455" s="5">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="T455" s="3" t="s">
         <v>1139</v>
@@ -61040,7 +61040,7 @@
         <v>46</v>
       </c>
       <c r="AA455" s="7">
-        <v>18082468</v>
+        <v>7870700</v>
       </c>
       <c r="AB455" s="7">
         <v>31</v>
@@ -61111,37 +61111,37 @@
         <v>1160</v>
       </c>
       <c r="I456" s="3" t="s">
-        <v>1185</v>
+        <v>170</v>
       </c>
       <c r="J456" s="3" t="s">
-        <v>1186</v>
+        <v>171</v>
       </c>
       <c r="K456" s="3" t="s">
-        <v>560</v>
+        <v>172</v>
       </c>
       <c r="L456" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M456" s="3" t="s">
-        <v>229</v>
+        <v>76</v>
       </c>
       <c r="N456" s="3" t="s">
-        <v>230</v>
+        <v>77</v>
       </c>
       <c r="O456" s="3" t="s">
-        <v>231</v>
+        <v>78</v>
       </c>
       <c r="P456" s="3" t="s">
-        <v>232</v>
+        <v>79</v>
       </c>
       <c r="Q456" s="5">
-        <v>4</v>
-      </c>
-      <c r="R456" s="3">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="R456" s="5">
+        <v>26</v>
       </c>
       <c r="S456" s="5">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="T456" s="3" t="s">
         <v>1139</v>
@@ -61165,7 +61165,7 @@
         <v>46</v>
       </c>
       <c r="AA456" s="7">
-        <v>379200</v>
+        <v>2196976</v>
       </c>
       <c r="AB456" s="7">
         <v>31</v>
@@ -61236,37 +61236,37 @@
         <v>1160</v>
       </c>
       <c r="I457" s="3" t="s">
-        <v>141</v>
+        <v>1185</v>
       </c>
       <c r="J457" s="3" t="s">
-        <v>142</v>
+        <v>1186</v>
       </c>
       <c r="K457" s="3" t="s">
-        <v>143</v>
+        <v>1187</v>
       </c>
       <c r="L457" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M457" s="3" t="s">
-        <v>62</v>
+        <v>161</v>
       </c>
       <c r="N457" s="3" t="s">
-        <v>63</v>
+        <v>162</v>
       </c>
       <c r="O457" s="3" t="s">
-        <v>64</v>
+        <v>163</v>
       </c>
       <c r="P457" s="3" t="s">
-        <v>65</v>
+        <v>164</v>
       </c>
       <c r="Q457" s="5">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="R457" s="5">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="S457" s="5">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="T457" s="3" t="s">
         <v>1139</v>
@@ -61290,7 +61290,7 @@
         <v>46</v>
       </c>
       <c r="AA457" s="7">
-        <v>7870700</v>
+        <v>1330200</v>
       </c>
       <c r="AB457" s="7">
         <v>31</v>
@@ -61361,37 +61361,37 @@
         <v>1160</v>
       </c>
       <c r="I458" s="3" t="s">
-        <v>170</v>
+        <v>269</v>
       </c>
       <c r="J458" s="3" t="s">
-        <v>171</v>
+        <v>270</v>
       </c>
       <c r="K458" s="3" t="s">
-        <v>172</v>
+        <v>271</v>
       </c>
       <c r="L458" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M458" s="3" t="s">
-        <v>76</v>
+        <v>137</v>
       </c>
       <c r="N458" s="3" t="s">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="O458" s="3" t="s">
-        <v>78</v>
+        <v>139</v>
       </c>
       <c r="P458" s="3" t="s">
-        <v>79</v>
+        <v>140</v>
       </c>
       <c r="Q458" s="5">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="R458" s="5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="S458" s="5">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="T458" s="3" t="s">
         <v>1139</v>
@@ -61415,7 +61415,7 @@
         <v>46</v>
       </c>
       <c r="AA458" s="7">
-        <v>2196976</v>
+        <v>16986149</v>
       </c>
       <c r="AB458" s="7">
         <v>31</v>
@@ -61486,13 +61486,13 @@
         <v>1160</v>
       </c>
       <c r="I459" s="3" t="s">
-        <v>1187</v>
+        <v>305</v>
       </c>
       <c r="J459" s="3" t="s">
-        <v>1188</v>
+        <v>306</v>
       </c>
       <c r="K459" s="3" t="s">
-        <v>1189</v>
+        <v>307</v>
       </c>
       <c r="L459" s="3" t="s">
         <v>50</v>
@@ -61510,13 +61510,13 @@
         <v>164</v>
       </c>
       <c r="Q459" s="5">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="R459" s="5">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="S459" s="5">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="T459" s="3" t="s">
         <v>1139</v>
@@ -61540,7 +61540,7 @@
         <v>46</v>
       </c>
       <c r="AA459" s="7">
-        <v>1330200</v>
+        <v>18082468</v>
       </c>
       <c r="AB459" s="7">
         <v>31</v>
@@ -61611,37 +61611,37 @@
         <v>1160</v>
       </c>
       <c r="I460" s="3" t="s">
-        <v>269</v>
+        <v>1188</v>
       </c>
       <c r="J460" s="3" t="s">
-        <v>270</v>
+        <v>1189</v>
       </c>
       <c r="K460" s="3" t="s">
-        <v>271</v>
+        <v>560</v>
       </c>
       <c r="L460" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M460" s="3" t="s">
-        <v>137</v>
+        <v>229</v>
       </c>
       <c r="N460" s="3" t="s">
-        <v>138</v>
+        <v>230</v>
       </c>
       <c r="O460" s="3" t="s">
-        <v>139</v>
+        <v>231</v>
       </c>
       <c r="P460" s="3" t="s">
-        <v>140</v>
+        <v>232</v>
       </c>
       <c r="Q460" s="5">
-        <v>14</v>
-      </c>
-      <c r="R460" s="5">
-        <v>12</v>
+        <v>4</v>
+      </c>
+      <c r="R460" s="3">
+        <v>0</v>
       </c>
       <c r="S460" s="5">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="T460" s="3" t="s">
         <v>1139</v>
@@ -61665,7 +61665,7 @@
         <v>46</v>
       </c>
       <c r="AA460" s="7">
-        <v>16001949</v>
+        <v>379200</v>
       </c>
       <c r="AB460" s="7">
         <v>31</v>
@@ -61861,13 +61861,13 @@
         <v>1160</v>
       </c>
       <c r="I462" s="3" t="s">
-        <v>1172</v>
+        <v>1167</v>
       </c>
       <c r="J462" s="3" t="s">
-        <v>1173</v>
+        <v>1168</v>
       </c>
       <c r="K462" s="3" t="s">
-        <v>1174</v>
+        <v>1169</v>
       </c>
       <c r="L462" s="3" t="s">
         <v>50</v>
@@ -62736,37 +62736,37 @@
         <v>1202</v>
       </c>
       <c r="I469" s="3" t="s">
-        <v>1203</v>
+        <v>1164</v>
       </c>
       <c r="J469" s="3" t="s">
-        <v>1204</v>
+        <v>1165</v>
       </c>
       <c r="K469" s="3" t="s">
-        <v>1205</v>
+        <v>1166</v>
       </c>
       <c r="L469" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M469" s="3" t="s">
-        <v>137</v>
+        <v>207</v>
       </c>
       <c r="N469" s="3" t="s">
-        <v>138</v>
+        <v>208</v>
       </c>
       <c r="O469" s="3" t="s">
-        <v>139</v>
+        <v>209</v>
       </c>
       <c r="P469" s="3" t="s">
-        <v>140</v>
+        <v>210</v>
       </c>
       <c r="Q469" s="5">
-        <v>6</v>
-      </c>
-      <c r="R469" s="3">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="R469" s="5">
+        <v>10</v>
       </c>
       <c r="S469" s="5">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="T469" s="3" t="s">
         <v>1139</v>
@@ -62790,7 +62790,7 @@
         <v>46</v>
       </c>
       <c r="AA469" s="7">
-        <v>2324385</v>
+        <v>848501</v>
       </c>
       <c r="AB469" s="7">
         <v>31</v>
@@ -62861,37 +62861,37 @@
         <v>1202</v>
       </c>
       <c r="I470" s="3" t="s">
-        <v>1164</v>
+        <v>1203</v>
       </c>
       <c r="J470" s="3" t="s">
-        <v>1165</v>
+        <v>1204</v>
       </c>
       <c r="K470" s="3" t="s">
-        <v>1166</v>
+        <v>1205</v>
       </c>
       <c r="L470" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M470" s="3" t="s">
-        <v>207</v>
+        <v>137</v>
       </c>
       <c r="N470" s="3" t="s">
-        <v>208</v>
+        <v>138</v>
       </c>
       <c r="O470" s="3" t="s">
-        <v>209</v>
+        <v>139</v>
       </c>
       <c r="P470" s="3" t="s">
-        <v>210</v>
+        <v>140</v>
       </c>
       <c r="Q470" s="5">
-        <v>10</v>
-      </c>
-      <c r="R470" s="5">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="R470" s="3">
+        <v>0</v>
       </c>
       <c r="S470" s="5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="T470" s="3" t="s">
         <v>1139</v>
@@ -62915,7 +62915,7 @@
         <v>46</v>
       </c>
       <c r="AA470" s="7">
-        <v>848501</v>
+        <v>2324385</v>
       </c>
       <c r="AB470" s="7">
         <v>31</v>
@@ -62986,13 +62986,13 @@
         <v>1160</v>
       </c>
       <c r="I471" s="3" t="s">
+        <v>1185</v>
+      </c>
+      <c r="J471" s="3" t="s">
+        <v>1186</v>
+      </c>
+      <c r="K471" s="3" t="s">
         <v>1187</v>
-      </c>
-      <c r="J471" s="3" t="s">
-        <v>1188</v>
-      </c>
-      <c r="K471" s="3" t="s">
-        <v>1189</v>
       </c>
       <c r="L471" s="3" t="s">
         <v>50</v>
@@ -63486,13 +63486,13 @@
         <v>1160</v>
       </c>
       <c r="I475" s="3" t="s">
-        <v>1172</v>
+        <v>1167</v>
       </c>
       <c r="J475" s="3" t="s">
-        <v>1173</v>
+        <v>1168</v>
       </c>
       <c r="K475" s="3" t="s">
-        <v>1174</v>
+        <v>1169</v>
       </c>
       <c r="L475" s="3" t="s">
         <v>50</v>
@@ -64915,7 +64915,7 @@
         <v>46</v>
       </c>
       <c r="AA486" s="7">
-        <v>8994825</v>
+        <v>9864825</v>
       </c>
       <c r="AB486" s="7">
         <v>1</v>
@@ -66415,7 +66415,7 @@
         <v>46</v>
       </c>
       <c r="AA498" s="7">
-        <v>471000</v>
+        <v>597118</v>
       </c>
       <c r="AB498" s="7">
         <v>1</v>
@@ -68915,7 +68915,7 @@
         <v>46</v>
       </c>
       <c r="AA518" s="7">
-        <v>710000</v>
+        <v>902000</v>
       </c>
       <c r="AB518" s="7">
         <v>31</v>
@@ -69111,13 +69111,13 @@
         <v>45</v>
       </c>
       <c r="I520" s="3" t="s">
-        <v>1172</v>
+        <v>1167</v>
       </c>
       <c r="J520" s="3" t="s">
-        <v>1173</v>
+        <v>1168</v>
       </c>
       <c r="K520" s="3" t="s">
-        <v>1174</v>
+        <v>1169</v>
       </c>
       <c r="L520" s="3" t="s">
         <v>50</v>
@@ -69361,13 +69361,13 @@
         <v>45</v>
       </c>
       <c r="I522" s="3" t="s">
-        <v>1167</v>
+        <v>1170</v>
       </c>
       <c r="J522" s="3" t="s">
-        <v>1168</v>
+        <v>1171</v>
       </c>
       <c r="K522" s="3" t="s">
-        <v>1169</v>
+        <v>1172</v>
       </c>
       <c r="L522" s="3" t="s">
         <v>50</v>
@@ -70885,13 +70885,13 @@
         <v>79</v>
       </c>
       <c r="Q534" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R534" s="5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="S534" s="5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="T534" s="3" t="s">
         <v>1139</v>
@@ -71361,13 +71361,13 @@
         <v>1160</v>
       </c>
       <c r="I538" s="3" t="s">
-        <v>1172</v>
+        <v>1167</v>
       </c>
       <c r="J538" s="3" t="s">
-        <v>1173</v>
+        <v>1168</v>
       </c>
       <c r="K538" s="3" t="s">
-        <v>1174</v>
+        <v>1169</v>
       </c>
       <c r="L538" s="3" t="s">
         <v>50</v>
@@ -71611,37 +71611,37 @@
         <v>1160</v>
       </c>
       <c r="I540" s="3" t="s">
-        <v>638</v>
+        <v>1052</v>
       </c>
       <c r="J540" s="3" t="s">
-        <v>639</v>
+        <v>1053</v>
       </c>
       <c r="K540" s="3" t="s">
-        <v>640</v>
+        <v>1054</v>
       </c>
       <c r="L540" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M540" s="3" t="s">
-        <v>147</v>
+        <v>62</v>
       </c>
       <c r="N540" s="3" t="s">
-        <v>148</v>
+        <v>63</v>
       </c>
       <c r="O540" s="3" t="s">
-        <v>149</v>
+        <v>64</v>
       </c>
       <c r="P540" s="3" t="s">
-        <v>150</v>
+        <v>65</v>
       </c>
       <c r="Q540" s="5">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="R540" s="5">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="S540" s="5">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="T540" s="3" t="s">
         <v>1139</v>
@@ -71665,7 +71665,7 @@
         <v>46</v>
       </c>
       <c r="AA540" s="7">
-        <v>2734208</v>
+        <v>672100</v>
       </c>
       <c r="AB540" s="7">
         <v>31</v>
@@ -71736,37 +71736,37 @@
         <v>1160</v>
       </c>
       <c r="I541" s="3" t="s">
-        <v>1277</v>
+        <v>638</v>
       </c>
       <c r="J541" s="3" t="s">
-        <v>1278</v>
+        <v>639</v>
       </c>
       <c r="K541" s="3" t="s">
-        <v>1279</v>
+        <v>640</v>
       </c>
       <c r="L541" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M541" s="3" t="s">
-        <v>193</v>
+        <v>147</v>
       </c>
       <c r="N541" s="3" t="s">
-        <v>194</v>
+        <v>148</v>
       </c>
       <c r="O541" s="3" t="s">
-        <v>195</v>
+        <v>149</v>
       </c>
       <c r="P541" s="3" t="s">
-        <v>196</v>
+        <v>150</v>
       </c>
       <c r="Q541" s="5">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="R541" s="5">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="S541" s="5">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="T541" s="3" t="s">
         <v>1139</v>
@@ -71790,7 +71790,7 @@
         <v>46</v>
       </c>
       <c r="AA541" s="7">
-        <v>1880508</v>
+        <v>2734208</v>
       </c>
       <c r="AB541" s="7">
         <v>31</v>
@@ -71861,37 +71861,37 @@
         <v>1160</v>
       </c>
       <c r="I542" s="3" t="s">
-        <v>660</v>
+        <v>1277</v>
       </c>
       <c r="J542" s="3" t="s">
-        <v>661</v>
+        <v>1278</v>
       </c>
       <c r="K542" s="3" t="s">
-        <v>662</v>
+        <v>1279</v>
       </c>
       <c r="L542" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M542" s="3" t="s">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="N542" s="3" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="O542" s="3" t="s">
-        <v>156</v>
+        <v>195</v>
       </c>
       <c r="P542" s="3" t="s">
-        <v>157</v>
+        <v>196</v>
       </c>
       <c r="Q542" s="5">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="R542" s="5">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="S542" s="5">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="T542" s="3" t="s">
         <v>1139</v>
@@ -71915,7 +71915,7 @@
         <v>46</v>
       </c>
       <c r="AA542" s="7">
-        <v>1218465</v>
+        <v>1880508</v>
       </c>
       <c r="AB542" s="7">
         <v>31</v>
@@ -71986,34 +71986,34 @@
         <v>1160</v>
       </c>
       <c r="I543" s="3" t="s">
-        <v>684</v>
+        <v>660</v>
       </c>
       <c r="J543" s="3" t="s">
-        <v>685</v>
+        <v>661</v>
       </c>
       <c r="K543" s="3" t="s">
-        <v>686</v>
+        <v>662</v>
       </c>
       <c r="L543" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M543" s="3" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="N543" s="3" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="O543" s="3" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="P543" s="3" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="Q543" s="5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R543" s="5">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="S543" s="5">
         <v>13</v>
@@ -72039,8 +72039,8 @@
       <c r="Z543" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA543" s="3" t="s">
-        <v>46</v>
+      <c r="AA543" s="7">
+        <v>1218465</v>
       </c>
       <c r="AB543" s="7">
         <v>31</v>
@@ -72111,37 +72111,37 @@
         <v>1160</v>
       </c>
       <c r="I544" s="3" t="s">
-        <v>1199</v>
+        <v>684</v>
       </c>
       <c r="J544" s="3" t="s">
-        <v>1200</v>
+        <v>685</v>
       </c>
       <c r="K544" s="3" t="s">
-        <v>1201</v>
+        <v>686</v>
       </c>
       <c r="L544" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M544" s="3" t="s">
-        <v>193</v>
+        <v>147</v>
       </c>
       <c r="N544" s="3" t="s">
-        <v>194</v>
+        <v>148</v>
       </c>
       <c r="O544" s="3" t="s">
-        <v>195</v>
+        <v>149</v>
       </c>
       <c r="P544" s="3" t="s">
-        <v>196</v>
+        <v>150</v>
       </c>
       <c r="Q544" s="5">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="R544" s="5">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="S544" s="5">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="T544" s="3" t="s">
         <v>1139</v>
@@ -72164,8 +72164,8 @@
       <c r="Z544" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA544" s="7">
-        <v>1507880</v>
+      <c r="AA544" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="AB544" s="7">
         <v>31</v>
@@ -72236,37 +72236,37 @@
         <v>1160</v>
       </c>
       <c r="I545" s="3" t="s">
-        <v>1052</v>
+        <v>1199</v>
       </c>
       <c r="J545" s="3" t="s">
-        <v>1053</v>
+        <v>1200</v>
       </c>
       <c r="K545" s="3" t="s">
-        <v>1054</v>
+        <v>1201</v>
       </c>
       <c r="L545" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M545" s="3" t="s">
-        <v>62</v>
+        <v>193</v>
       </c>
       <c r="N545" s="3" t="s">
-        <v>63</v>
+        <v>194</v>
       </c>
       <c r="O545" s="3" t="s">
-        <v>64</v>
+        <v>195</v>
       </c>
       <c r="P545" s="3" t="s">
-        <v>65</v>
+        <v>196</v>
       </c>
       <c r="Q545" s="5">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="R545" s="5">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="S545" s="5">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="T545" s="3" t="s">
         <v>1139</v>
@@ -72290,7 +72290,7 @@
         <v>46</v>
       </c>
       <c r="AA545" s="7">
-        <v>672100</v>
+        <v>1507880</v>
       </c>
       <c r="AB545" s="7">
         <v>31</v>
@@ -72361,37 +72361,37 @@
         <v>1287</v>
       </c>
       <c r="I546" s="3" t="s">
-        <v>614</v>
+        <v>1075</v>
       </c>
       <c r="J546" s="3" t="s">
-        <v>615</v>
+        <v>1076</v>
       </c>
       <c r="K546" s="3" t="s">
-        <v>616</v>
+        <v>1077</v>
       </c>
       <c r="L546" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M546" s="3" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="N546" s="3" t="s">
-        <v>162</v>
+        <v>138</v>
       </c>
       <c r="O546" s="3" t="s">
-        <v>163</v>
+        <v>139</v>
       </c>
       <c r="P546" s="3" t="s">
-        <v>164</v>
+        <v>140</v>
       </c>
       <c r="Q546" s="5">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="R546" s="5">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="S546" s="5">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="T546" s="3" t="s">
         <v>1139</v>
@@ -72415,7 +72415,7 @@
         <v>46</v>
       </c>
       <c r="AA546" s="7">
-        <v>3741248</v>
+        <v>4678207</v>
       </c>
       <c r="AB546" s="7">
         <v>31</v>
@@ -72486,37 +72486,37 @@
         <v>1287</v>
       </c>
       <c r="I547" s="3" t="s">
-        <v>1075</v>
+        <v>614</v>
       </c>
       <c r="J547" s="3" t="s">
-        <v>1076</v>
+        <v>615</v>
       </c>
       <c r="K547" s="3" t="s">
-        <v>1077</v>
+        <v>616</v>
       </c>
       <c r="L547" s="3" t="s">
         <v>50</v>
       </c>
       <c r="M547" s="3" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="N547" s="3" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="O547" s="3" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="P547" s="3" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="Q547" s="5">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="R547" s="5">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="S547" s="5">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="T547" s="3" t="s">
         <v>1139</v>
@@ -72540,7 +72540,7 @@
         <v>46</v>
       </c>
       <c r="AA547" s="7">
-        <v>4678207</v>
+        <v>3741248</v>
       </c>
       <c r="AB547" s="7">
         <v>31</v>
@@ -75111,13 +75111,13 @@
         <v>45</v>
       </c>
       <c r="I568" s="3" t="s">
-        <v>1172</v>
+        <v>1167</v>
       </c>
       <c r="J568" s="3" t="s">
-        <v>1173</v>
+        <v>1168</v>
       </c>
       <c r="K568" s="3" t="s">
-        <v>1174</v>
+        <v>1169</v>
       </c>
       <c r="L568" s="3" t="s">
         <v>50</v>
@@ -75665,7 +75665,7 @@
         <v>46</v>
       </c>
       <c r="AA572" s="7">
-        <v>1407238</v>
+        <v>1867238</v>
       </c>
       <c r="AB572" s="7">
         <v>31</v>
@@ -76415,7 +76415,7 @@
         <v>46</v>
       </c>
       <c r="AA578" s="7">
-        <v>3163624</v>
+        <v>5198074</v>
       </c>
       <c r="AB578" s="7">
         <v>31</v>
@@ -77289,8 +77289,8 @@
       <c r="Z585" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AA585" s="3" t="s">
-        <v>46</v>
+      <c r="AA585" s="7">
+        <v>156000</v>
       </c>
       <c r="AB585" s="7">
         <v>31</v>
@@ -77540,7 +77540,7 @@
         <v>46</v>
       </c>
       <c r="AA587" s="7">
-        <v>455000</v>
+        <v>762981</v>
       </c>
       <c r="AB587" s="7">
         <v>31</v>

</xml_diff>